<commit_message>
xử lý ngày chủ nhật và tên ca
</commit_message>
<xml_diff>
--- a/convert/data1.xlsx
+++ b/convert/data1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28192" uniqueCount="801">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28148" uniqueCount="801">
   <si>
     <t>Công ty TNHH Sản Xuất Hiệp Phước Thành</t>
   </si>
@@ -17993,32 +17993,35 @@
       <c r="Z171" t="s">
         <v>49</v>
       </c>
-      <c r="AB171" t="s">
-        <v>83</v>
-      </c>
-      <c r="AC171" t="s">
-        <v>49</v>
-      </c>
-      <c r="AD171" t="s">
-        <v>49</v>
-      </c>
-      <c r="AE171" t="s">
-        <v>51</v>
-      </c>
-      <c r="AF171" t="s">
-        <v>49</v>
-      </c>
-      <c r="AG171" t="s">
-        <v>49</v>
-      </c>
-      <c r="AH171" t="s">
-        <v>49</v>
-      </c>
-      <c r="AI171" t="s">
-        <v>49</v>
+      <c r="AA171">
+        <v>34</v>
+      </c>
+      <c r="AB171">
+        <v>1</v>
+      </c>
+      <c r="AC171">
+        <v>0</v>
+      </c>
+      <c r="AD171">
+        <v>0</v>
+      </c>
+      <c r="AE171">
+        <v>19.4</v>
+      </c>
+      <c r="AF171">
+        <v>0</v>
+      </c>
+      <c r="AG171">
+        <v>0</v>
+      </c>
+      <c r="AH171">
+        <v>0</v>
+      </c>
+      <c r="AI171">
+        <v>0</v>
       </c>
       <c r="AJ171">
-        <v>12</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="172" spans="1:37">
@@ -25756,29 +25759,35 @@
       <c r="Z256" t="s">
         <v>49</v>
       </c>
-      <c r="AC256" t="s">
-        <v>49</v>
-      </c>
-      <c r="AD256" t="s">
-        <v>49</v>
-      </c>
-      <c r="AE256" t="s">
-        <v>51</v>
-      </c>
-      <c r="AF256" t="s">
-        <v>49</v>
-      </c>
-      <c r="AG256" t="s">
-        <v>49</v>
-      </c>
-      <c r="AH256" t="s">
-        <v>49</v>
-      </c>
-      <c r="AI256" t="s">
-        <v>49</v>
+      <c r="AA256">
+        <v>0</v>
+      </c>
+      <c r="AB256">
+        <v>0</v>
+      </c>
+      <c r="AC256">
+        <v>0</v>
+      </c>
+      <c r="AD256">
+        <v>0</v>
+      </c>
+      <c r="AE256">
+        <v>20</v>
+      </c>
+      <c r="AF256">
+        <v>0</v>
+      </c>
+      <c r="AG256">
+        <v>0</v>
+      </c>
+      <c r="AH256">
+        <v>0</v>
+      </c>
+      <c r="AI256">
+        <v>0</v>
       </c>
       <c r="AJ256">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="257" spans="1:37">
@@ -48717,29 +48726,35 @@
       <c r="Z509" t="s">
         <v>49</v>
       </c>
-      <c r="AC509" t="s">
-        <v>49</v>
-      </c>
-      <c r="AD509" t="s">
-        <v>49</v>
-      </c>
-      <c r="AE509" t="s">
-        <v>51</v>
-      </c>
-      <c r="AF509" t="s">
-        <v>49</v>
-      </c>
-      <c r="AG509" t="s">
-        <v>49</v>
-      </c>
-      <c r="AH509" t="s">
-        <v>49</v>
-      </c>
-      <c r="AI509" t="s">
-        <v>49</v>
+      <c r="AA509">
+        <v>0</v>
+      </c>
+      <c r="AB509">
+        <v>0</v>
+      </c>
+      <c r="AC509">
+        <v>0</v>
+      </c>
+      <c r="AD509">
+        <v>0</v>
+      </c>
+      <c r="AE509">
+        <v>20</v>
+      </c>
+      <c r="AF509">
+        <v>0</v>
+      </c>
+      <c r="AG509">
+        <v>0</v>
+      </c>
+      <c r="AH509">
+        <v>0</v>
+      </c>
+      <c r="AI509">
+        <v>0</v>
       </c>
       <c r="AJ509">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="510" spans="1:37">
@@ -58684,29 +58699,35 @@
       <c r="Z622" t="s">
         <v>49</v>
       </c>
-      <c r="AC622" t="s">
-        <v>49</v>
-      </c>
-      <c r="AD622" t="s">
-        <v>49</v>
-      </c>
-      <c r="AE622" t="s">
-        <v>51</v>
-      </c>
-      <c r="AF622" t="s">
-        <v>49</v>
-      </c>
-      <c r="AG622" t="s">
-        <v>49</v>
-      </c>
-      <c r="AH622" t="s">
-        <v>49</v>
-      </c>
-      <c r="AI622" t="s">
-        <v>49</v>
+      <c r="AA622">
+        <v>0</v>
+      </c>
+      <c r="AB622">
+        <v>0</v>
+      </c>
+      <c r="AC622">
+        <v>0</v>
+      </c>
+      <c r="AD622">
+        <v>0</v>
+      </c>
+      <c r="AE622">
+        <v>20</v>
+      </c>
+      <c r="AF622">
+        <v>0</v>
+      </c>
+      <c r="AG622">
+        <v>0</v>
+      </c>
+      <c r="AH622">
+        <v>0</v>
+      </c>
+      <c r="AI622">
+        <v>0</v>
       </c>
       <c r="AJ622">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="623" spans="1:37">
@@ -75349,29 +75370,35 @@
       <c r="Z811" t="s">
         <v>49</v>
       </c>
-      <c r="AC811" t="s">
-        <v>49</v>
-      </c>
-      <c r="AD811" t="s">
-        <v>49</v>
-      </c>
-      <c r="AE811" t="s">
-        <v>51</v>
-      </c>
-      <c r="AF811" t="s">
-        <v>49</v>
-      </c>
-      <c r="AG811" t="s">
-        <v>49</v>
-      </c>
-      <c r="AH811" t="s">
-        <v>49</v>
-      </c>
-      <c r="AI811" t="s">
-        <v>49</v>
+      <c r="AA811">
+        <v>0</v>
+      </c>
+      <c r="AB811">
+        <v>0</v>
+      </c>
+      <c r="AC811">
+        <v>0</v>
+      </c>
+      <c r="AD811">
+        <v>0</v>
+      </c>
+      <c r="AE811">
+        <v>20</v>
+      </c>
+      <c r="AF811">
+        <v>0</v>
+      </c>
+      <c r="AG811">
+        <v>0</v>
+      </c>
+      <c r="AH811">
+        <v>0</v>
+      </c>
+      <c r="AI811">
+        <v>0</v>
       </c>
       <c r="AJ811">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="812" spans="1:37">
@@ -90116,29 +90143,32 @@
       <c r="Z975" t="s">
         <v>49</v>
       </c>
-      <c r="AB975" t="s">
-        <v>83</v>
-      </c>
-      <c r="AC975" t="s">
-        <v>49</v>
-      </c>
-      <c r="AD975" t="s">
-        <v>49</v>
-      </c>
-      <c r="AE975" t="s">
-        <v>51</v>
-      </c>
-      <c r="AF975" t="s">
-        <v>49</v>
-      </c>
-      <c r="AG975" t="s">
-        <v>49</v>
-      </c>
-      <c r="AH975" t="s">
-        <v>49</v>
-      </c>
-      <c r="AI975" t="s">
-        <v>49</v>
+      <c r="AA975">
+        <v>0</v>
+      </c>
+      <c r="AB975">
+        <v>1</v>
+      </c>
+      <c r="AC975">
+        <v>8</v>
+      </c>
+      <c r="AD975">
+        <v>0</v>
+      </c>
+      <c r="AE975">
+        <v>12</v>
+      </c>
+      <c r="AF975">
+        <v>0</v>
+      </c>
+      <c r="AG975">
+        <v>0</v>
+      </c>
+      <c r="AH975">
+        <v>0</v>
+      </c>
+      <c r="AI975">
+        <v>0</v>
       </c>
       <c r="AJ975">
         <v>12</v>

</xml_diff>